<commit_message>
Fixed user logout option not appearing in thank you page
</commit_message>
<xml_diff>
--- a/documentation/Tests.xlsx
+++ b/documentation/Tests.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://collyer82-my.sharepoint.com/personal/25cookeg899_collyers_ac_uk/Documents/01 - Computer Science/Python Projects/Theatre-Booking/documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="119" documentId="8_{8A25BE57-B96B-4758-82AD-3B4D19E7B08C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6D1FE015-43A9-443E-A62D-94B268B67299}"/>
+  <xr:revisionPtr revIDLastSave="219" documentId="8_{8A25BE57-B96B-4758-82AD-3B4D19E7B08C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E908D8FB-0E5E-4CB0-A919-19C0E4747D78}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{0216B08E-6C11-4E2A-9B97-BB4BC5AB6A5B}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="121">
   <si>
     <t>Test No</t>
   </si>
@@ -212,9 +212,6 @@
     <t>Check users button redirect from admin add performance page works</t>
   </si>
   <si>
-    <t>Check dhasboard button redirect from add performance page.</t>
-  </si>
-  <si>
     <t>Press dashboard in the nav bar of add performance page.</t>
   </si>
   <si>
@@ -225,6 +222,186 @@
   </si>
   <si>
     <t>Press ADMIN in nav bar of add perormance page.</t>
+  </si>
+  <si>
+    <t>Add valid data to all fields in admin add performance</t>
+  </si>
+  <si>
+    <t>Check admin add performance works with valid data (w/ description, no unavailable seats)</t>
+  </si>
+  <si>
+    <t>Check admin add performance works with valid data (no description, no unavailable seats)</t>
+  </si>
+  <si>
+    <t>Add valid data to all fields in admin add performance except for description</t>
+  </si>
+  <si>
+    <t>Performance is added to database and user is redirected to admin dashbaord with new performance visible.</t>
+  </si>
+  <si>
+    <t>Check admin add performance works with valid data (w/ description, w/ unavailable seats)</t>
+  </si>
+  <si>
+    <t>Add valid data to all fields in admin add performance and mark seats as unavailable.</t>
+  </si>
+  <si>
+    <t>Performance is added to database  as well as unavailable seats and user is redirected to admin dashbaord with new performance visible.</t>
+  </si>
+  <si>
+    <t>Check add performacne works with no title.</t>
+  </si>
+  <si>
+    <t>Do not add title to add performacne page.</t>
+  </si>
+  <si>
+    <t>Flash message appears, data it not added to database and user is not redirected.</t>
+  </si>
+  <si>
+    <t>Check add performance works with no price.</t>
+  </si>
+  <si>
+    <t>Delete prices from add performance (also add title)</t>
+  </si>
+  <si>
+    <t>Delete prices from add performance and try to type a letter.</t>
+  </si>
+  <si>
+    <t>Letter cannot be typed.</t>
+  </si>
+  <si>
+    <t>Check performance works when trying to type letter in price field.</t>
+  </si>
+  <si>
+    <t>Check performance works with boundary length title.</t>
+  </si>
+  <si>
+    <t>Type title that is 100 characters long.</t>
+  </si>
+  <si>
+    <t>Type title that is 101 characters long.</t>
+  </si>
+  <si>
+    <t>Flash message is show, data is not added to database, user is not redirected.</t>
+  </si>
+  <si>
+    <t>Check add performance works with invalid length title.</t>
+  </si>
+  <si>
+    <t>Check dashboard button redirect from add performance page.</t>
+  </si>
+  <si>
+    <t>Check add showing button works with adding showing from previous date</t>
+  </si>
+  <si>
+    <t>Set date o fperformance to date in the past</t>
+  </si>
+  <si>
+    <t>Flash message appears saying date is in the past and nothing is added to DB</t>
+  </si>
+  <si>
+    <t>Check add showing works with valid date</t>
+  </si>
+  <si>
+    <t>Set date of performance to date in future</t>
+  </si>
+  <si>
+    <t>Showing is added to DB, page refreshes, new showing appears (empty of bookings and with valid revenue (£0))</t>
+  </si>
+  <si>
+    <t>Check add showing works with boundary date</t>
+  </si>
+  <si>
+    <t>Set date of showing to today</t>
+  </si>
+  <si>
+    <t>Check delete showing button works</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Click delete showing button </t>
+  </si>
+  <si>
+    <t>Check delete performance button works</t>
+  </si>
+  <si>
+    <t>Click delete performance button</t>
+  </si>
+  <si>
+    <t>Performance is deleted with all showings and bookings associated with it.</t>
+  </si>
+  <si>
+    <t>Showing is deleted with all bookings associated with it from DB and page is refreshed</t>
+  </si>
+  <si>
+    <t>Check admin logout works in admin view users page</t>
+  </si>
+  <si>
+    <t>Check dashboard redirect works in admin view users page</t>
+  </si>
+  <si>
+    <t>Click dashboard in top left of admin users page</t>
+  </si>
+  <si>
+    <t>Redirect to admin dashbpard page</t>
+  </si>
+  <si>
+    <t>Click ADMIN in top right of nav bar in admin users page</t>
+  </si>
+  <si>
+    <t>Redirect to main login page</t>
+  </si>
+  <si>
+    <t>Check update user to SPECIAL works</t>
+  </si>
+  <si>
+    <t>Check update user to VISITOR works</t>
+  </si>
+  <si>
+    <t>Check update user to ADMIN works</t>
+  </si>
+  <si>
+    <t>Check update user to SPECIAL works from search</t>
+  </si>
+  <si>
+    <t>Check update user to VISITOR worksfrom search</t>
+  </si>
+  <si>
+    <t>Check update user to ADMIN worksfrom search</t>
+  </si>
+  <si>
+    <t>Check search works</t>
+  </si>
+  <si>
+    <t>Change user type to special</t>
+  </si>
+  <si>
+    <t>Change user type to visitor</t>
+  </si>
+  <si>
+    <t>Change user type to admin</t>
+  </si>
+  <si>
+    <t>Check delete user works</t>
+  </si>
+  <si>
+    <t>Delete user</t>
+  </si>
+  <si>
+    <t>Check delete user works from search</t>
+  </si>
+  <si>
+    <t>Search and update a user</t>
+  </si>
+  <si>
+    <t>Search and delete a user</t>
+  </si>
+  <si>
+    <t>Data is updated in DB and page is refreshed to represent</t>
+  </si>
+  <si>
+    <t>Relevent search results appear</t>
+  </si>
+  <si>
+    <t>Search in search bar</t>
   </si>
 </sst>
 </file>
@@ -282,32 +459,35 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="2">
     <dxf>
       <font>
         <color theme="9" tint="-0.499984740745262"/>
@@ -328,16 +508,6 @@
         </patternFill>
       </fill>
     </dxf>
-    <dxf>
-      <font>
-        <color theme="9" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -349,6 +519,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -668,2943 +842,3169 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7A683F2-5104-47AA-9E97-E0C89AF6B06D}">
-  <dimension ref="A1:G452"/>
+  <dimension ref="A1:G454"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.6640625" style="7" customWidth="1"/>
-    <col min="2" max="2" width="30.88671875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="33.77734375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="25.6640625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="29" style="1" customWidth="1"/>
-    <col min="6" max="6" width="12.6640625" style="6" customWidth="1"/>
-    <col min="7" max="7" width="63" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.88671875" style="1"/>
+    <col min="1" max="1" width="5.6640625" style="6" customWidth="1"/>
+    <col min="2" max="2" width="30.88671875" customWidth="1"/>
+    <col min="3" max="3" width="33.77734375" customWidth="1"/>
+    <col min="4" max="4" width="25.6640625" customWidth="1"/>
+    <col min="5" max="5" width="29" customWidth="1"/>
+    <col min="6" max="6" width="12.6640625" style="5" customWidth="1"/>
+    <col min="7" max="7" width="63" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:7" s="3" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="7">
+      <c r="A2" s="6">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="5"/>
+      <c r="F2" s="4"/>
     </row>
     <row r="3" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A3" s="7">
+      <c r="A3" s="6">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="5"/>
+      <c r="F3" s="4"/>
     </row>
     <row r="4" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A4" s="7">
+      <c r="A4" s="6">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="F4" s="5"/>
+      <c r="F4" s="4"/>
     </row>
     <row r="5" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="7">
+      <c r="A5" s="6">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="F5" s="5"/>
+      <c r="F5" s="4"/>
     </row>
     <row r="6" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A6" s="7">
+      <c r="A6" s="6">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F6" s="5"/>
+      <c r="F6" s="4"/>
     </row>
     <row r="7" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A7" s="7">
+      <c r="A7" s="6">
         <v>6</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="F7" s="5"/>
+      <c r="F7" s="4"/>
     </row>
     <row r="8" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A8" s="7">
+      <c r="A8" s="6">
         <v>7</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="1" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A9" s="7">
+      <c r="A9" s="6">
         <f>SUM(A8+1)</f>
         <v>8</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="1" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A10" s="7">
-        <f t="shared" ref="A10:A73" si="0">SUM(A9+1)</f>
+      <c r="A10" s="6">
+        <f t="shared" ref="A10:A75" si="0">SUM(A9+1)</f>
         <v>9</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="1" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="7">
+      <c r="A11" s="6">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="1" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A12" s="7">
+      <c r="A12" s="6">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="D12" s="1" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A13" s="7">
+      <c r="A13" s="6">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C13" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="D13" s="1" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A14" s="7">
+      <c r="A14" s="6">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="D14" s="1" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A15" s="7">
+      <c r="A15" s="6">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C15" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="D15" s="1" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A16" s="7">
+      <c r="A16" s="6">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="D16" s="1" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A17" s="7">
+      <c r="A17" s="6">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="C17" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="D17" s="1" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A18" s="7">
+      <c r="A18" s="6">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="C18" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="D18" s="1" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A19" s="7">
+      <c r="A19" s="6">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="C19" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="D19" s="1" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A20" s="7">
+      <c r="A20" s="6">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="C20" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="D20" s="2" t="s">
+      <c r="D20" s="1" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A21" s="7">
+      <c r="A21" s="6">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C21" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="D21" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A22" s="6">
+        <f t="shared" si="0"/>
+        <v>21</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C22" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="D21" s="2" t="s">
+      <c r="D22" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A23" s="6">
+        <f t="shared" si="0"/>
+        <v>22</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+      <c r="A24" s="6">
+        <f t="shared" si="0"/>
+        <v>23</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+      <c r="A25" s="6">
+        <f t="shared" si="0"/>
+        <v>24</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A26" s="6">
+        <f t="shared" si="0"/>
+        <v>25</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A27" s="6">
+        <f t="shared" si="0"/>
+        <v>26</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A28" s="6">
+        <f t="shared" si="0"/>
+        <v>27</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A29" s="6">
+        <f t="shared" si="0"/>
+        <v>28</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+      <c r="A30" s="6">
+        <f t="shared" si="0"/>
+        <v>29</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A31" s="6">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A32" s="6">
+        <f t="shared" si="0"/>
+        <v>31</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A33" s="6">
+        <f t="shared" si="0"/>
+        <v>32</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A34" s="6">
+        <f t="shared" si="0"/>
+        <v>33</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A35" s="6">
+        <f t="shared" si="0"/>
+        <v>34</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A36" s="6">
+        <f t="shared" si="0"/>
+        <v>35</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A37" s="6">
+        <f t="shared" si="0"/>
+        <v>36</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A38" s="6">
+        <f t="shared" si="0"/>
+        <v>37</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A39" s="6">
+        <f t="shared" si="0"/>
+        <v>38</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A40" s="6">
+        <f t="shared" si="0"/>
+        <v>39</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A41" s="6">
+        <f t="shared" si="0"/>
+        <v>40</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A42" s="6">
+        <v>40</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" s="8" customFormat="1" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="6">
+        <v>41</v>
+      </c>
+      <c r="B43" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="C43" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="D43" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="F43" s="5"/>
+    </row>
+    <row r="44" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A44" s="6">
+        <f>SUM(A43+1)</f>
+        <v>42</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A45" s="6">
+        <f t="shared" si="0"/>
+        <v>43</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A46" s="6">
+        <f t="shared" si="0"/>
+        <v>44</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A47" s="6">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A48" s="6">
+        <f t="shared" si="0"/>
+        <v>46</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A49" s="6">
+        <f t="shared" si="0"/>
+        <v>47</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A50" s="6">
+        <f t="shared" si="0"/>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A51" s="6">
+        <f t="shared" si="0"/>
+        <v>49</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A52" s="6">
+        <f t="shared" si="0"/>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A53" s="6">
+        <f t="shared" si="0"/>
         <v>51</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A22" s="7">
-        <f t="shared" si="0"/>
-        <v>21</v>
-      </c>
-      <c r="B22" s="2" t="s">
+    <row r="54" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A54" s="6">
+        <f t="shared" si="0"/>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A55" s="6">
+        <f t="shared" si="0"/>
+        <v>53</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A56" s="6">
+        <f t="shared" si="0"/>
+        <v>54</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A57" s="6">
+        <f t="shared" si="0"/>
+        <v>55</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A58" s="6">
+        <f t="shared" si="0"/>
         <v>56</v>
       </c>
-      <c r="C22" s="2" t="s">
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A59" s="6">
+        <f t="shared" si="0"/>
+        <v>57</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A60" s="6">
+        <f t="shared" si="0"/>
+        <v>58</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A61" s="6">
+        <f t="shared" si="0"/>
         <v>59</v>
       </c>
-      <c r="D22" s="2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A23" s="7">
-        <f t="shared" si="0"/>
-        <v>22</v>
-      </c>
-      <c r="B23" s="2" t="s">
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A62" s="6">
+        <f t="shared" si="0"/>
         <v>60</v>
       </c>
-      <c r="C23" s="2" t="s">
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A63" s="6">
+        <f t="shared" si="0"/>
         <v>61</v>
       </c>
-      <c r="D23" s="2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A24" s="7">
-        <f t="shared" si="0"/>
-        <v>23</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A25" s="7">
-        <f t="shared" si="0"/>
-        <v>24</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26" s="7">
-        <f t="shared" si="0"/>
-        <v>25</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A27" s="7">
-        <f t="shared" si="0"/>
-        <v>26</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A28" s="7">
-        <f t="shared" si="0"/>
-        <v>27</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A29" s="7">
-        <f t="shared" si="0"/>
-        <v>28</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A30" s="7">
-        <f t="shared" si="0"/>
-        <v>29</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A31" s="7">
-        <f t="shared" si="0"/>
-        <v>30</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A32" s="7">
-        <f t="shared" si="0"/>
-        <v>31</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A33" s="7">
-        <f t="shared" si="0"/>
-        <v>32</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A34" s="7">
-        <f t="shared" si="0"/>
-        <v>33</v>
-      </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A35" s="7">
-        <f t="shared" si="0"/>
-        <v>34</v>
-      </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A36" s="7">
-        <f t="shared" si="0"/>
-        <v>35</v>
-      </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A37" s="7">
-        <f t="shared" si="0"/>
-        <v>36</v>
-      </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A38" s="7">
-        <f t="shared" si="0"/>
-        <v>37</v>
-      </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A39" s="7">
-        <f t="shared" si="0"/>
-        <v>38</v>
-      </c>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A40" s="7">
-        <f t="shared" si="0"/>
-        <v>39</v>
-      </c>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A41" s="7">
-        <f t="shared" si="0"/>
-        <v>40</v>
-      </c>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A42" s="7">
-        <f t="shared" si="0"/>
-        <v>41</v>
-      </c>
-    </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A43" s="7">
-        <f t="shared" si="0"/>
-        <v>42</v>
-      </c>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A44" s="7">
-        <f t="shared" si="0"/>
-        <v>43</v>
-      </c>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A45" s="7">
-        <f t="shared" si="0"/>
-        <v>44</v>
-      </c>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A46" s="7">
-        <f t="shared" si="0"/>
-        <v>45</v>
-      </c>
-    </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A47" s="7">
-        <f t="shared" si="0"/>
-        <v>46</v>
-      </c>
-    </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A48" s="7">
-        <f t="shared" si="0"/>
-        <v>47</v>
-      </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A49" s="7">
-        <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A50" s="7">
-        <f t="shared" si="0"/>
-        <v>49</v>
-      </c>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A51" s="7">
-        <f t="shared" si="0"/>
-        <v>50</v>
-      </c>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A52" s="7">
-        <f t="shared" si="0"/>
-        <v>51</v>
-      </c>
-    </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A53" s="7">
-        <f t="shared" si="0"/>
-        <v>52</v>
-      </c>
-    </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A54" s="7">
-        <f t="shared" si="0"/>
-        <v>53</v>
-      </c>
-    </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A55" s="7">
-        <f t="shared" si="0"/>
-        <v>54</v>
-      </c>
-    </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A56" s="7">
-        <f t="shared" si="0"/>
-        <v>55</v>
-      </c>
-    </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A57" s="7">
-        <f t="shared" si="0"/>
-        <v>56</v>
-      </c>
-    </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A58" s="7">
-        <f t="shared" si="0"/>
-        <v>57</v>
-      </c>
-    </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A59" s="7">
-        <f t="shared" si="0"/>
-        <v>58</v>
-      </c>
-    </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A60" s="7">
-        <f t="shared" si="0"/>
-        <v>59</v>
-      </c>
-    </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A61" s="7">
-        <f t="shared" si="0"/>
-        <v>60</v>
-      </c>
-    </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A62" s="7">
-        <f t="shared" si="0"/>
-        <v>61</v>
-      </c>
-    </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A63" s="7">
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A64" s="6">
         <f t="shared" si="0"/>
         <v>62</v>
       </c>
     </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A64" s="7">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A65" s="6">
         <f t="shared" si="0"/>
         <v>63</v>
       </c>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A65" s="7">
+    <row r="66" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A66" s="6">
         <f t="shared" si="0"/>
         <v>64</v>
       </c>
     </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A66" s="7">
+    <row r="67" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A67" s="6">
         <f t="shared" si="0"/>
         <v>65</v>
       </c>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A67" s="7">
+    <row r="68" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A68" s="6">
         <f t="shared" si="0"/>
         <v>66</v>
       </c>
     </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A68" s="7">
+    <row r="69" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A69" s="6">
         <f t="shared" si="0"/>
         <v>67</v>
       </c>
     </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A69" s="7">
+    <row r="70" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A70" s="6">
         <f t="shared" si="0"/>
         <v>68</v>
       </c>
     </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A70" s="7">
+    <row r="71" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A71" s="6">
         <f t="shared" si="0"/>
         <v>69</v>
       </c>
     </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A71" s="7">
+    <row r="72" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A72" s="6">
         <f t="shared" si="0"/>
         <v>70</v>
       </c>
     </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A72" s="7">
+    <row r="73" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A73" s="6">
         <f t="shared" si="0"/>
         <v>71</v>
       </c>
     </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A73" s="7">
+    <row r="74" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A74" s="6">
         <f t="shared" si="0"/>
         <v>72</v>
       </c>
     </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A74" s="7">
-        <f t="shared" ref="A74:A137" si="1">SUM(A73+1)</f>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A75" s="6">
+        <f t="shared" si="0"/>
         <v>73</v>
       </c>
     </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A75" s="7">
-        <f t="shared" si="1"/>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A76" s="6">
+        <f t="shared" ref="A76:A139" si="1">SUM(A75+1)</f>
         <v>74</v>
       </c>
     </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A76" s="7">
+    <row r="77" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A77" s="6">
         <f t="shared" si="1"/>
         <v>75</v>
       </c>
     </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A77" s="7">
+    <row r="78" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A78" s="6">
         <f t="shared" si="1"/>
         <v>76</v>
       </c>
     </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A78" s="7">
+    <row r="79" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A79" s="6">
         <f t="shared" si="1"/>
         <v>77</v>
       </c>
     </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A79" s="7">
+    <row r="80" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A80" s="6">
         <f t="shared" si="1"/>
         <v>78</v>
       </c>
     </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A80" s="7">
+    <row r="81" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A81" s="6">
         <f t="shared" si="1"/>
         <v>79</v>
       </c>
     </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A81" s="7">
+    <row r="82" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A82" s="6">
         <f t="shared" si="1"/>
         <v>80</v>
       </c>
     </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A82" s="7">
+    <row r="83" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A83" s="6">
         <f t="shared" si="1"/>
         <v>81</v>
       </c>
     </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A83" s="7">
+    <row r="84" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A84" s="6">
         <f t="shared" si="1"/>
         <v>82</v>
       </c>
     </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A84" s="7">
+    <row r="85" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A85" s="6">
         <f t="shared" si="1"/>
         <v>83</v>
       </c>
     </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A85" s="7">
+    <row r="86" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A86" s="6">
         <f t="shared" si="1"/>
         <v>84</v>
       </c>
     </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A86" s="7">
+    <row r="87" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A87" s="6">
         <f t="shared" si="1"/>
         <v>85</v>
       </c>
     </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A87" s="7">
+    <row r="88" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A88" s="6">
         <f t="shared" si="1"/>
         <v>86</v>
       </c>
     </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A88" s="7">
+    <row r="89" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A89" s="6">
         <f t="shared" si="1"/>
         <v>87</v>
       </c>
     </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A89" s="7">
+    <row r="90" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A90" s="6">
         <f t="shared" si="1"/>
         <v>88</v>
       </c>
     </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A90" s="7">
+    <row r="91" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A91" s="6">
         <f t="shared" si="1"/>
         <v>89</v>
       </c>
     </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A91" s="7">
+    <row r="92" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A92" s="6">
         <f t="shared" si="1"/>
         <v>90</v>
       </c>
     </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A92" s="7">
+    <row r="93" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A93" s="6">
         <f t="shared" si="1"/>
         <v>91</v>
       </c>
     </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A93" s="7">
+    <row r="94" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A94" s="6">
         <f t="shared" si="1"/>
         <v>92</v>
       </c>
     </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A94" s="7">
+    <row r="95" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A95" s="6">
         <f t="shared" si="1"/>
         <v>93</v>
       </c>
     </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A95" s="7">
+    <row r="96" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A96" s="6">
         <f t="shared" si="1"/>
         <v>94</v>
       </c>
     </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A96" s="7">
+    <row r="97" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A97" s="6">
         <f t="shared" si="1"/>
         <v>95</v>
       </c>
     </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A97" s="7">
+    <row r="98" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A98" s="6">
         <f t="shared" si="1"/>
         <v>96</v>
       </c>
     </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A98" s="7">
+    <row r="99" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A99" s="6">
         <f t="shared" si="1"/>
         <v>97</v>
       </c>
     </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A99" s="7">
+    <row r="100" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A100" s="6">
         <f t="shared" si="1"/>
         <v>98</v>
       </c>
     </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A100" s="7">
+    <row r="101" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A101" s="6">
         <f t="shared" si="1"/>
         <v>99</v>
       </c>
     </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A101" s="7">
+    <row r="102" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A102" s="6">
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
     </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A102" s="7">
+    <row r="103" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A103" s="6">
         <f t="shared" si="1"/>
         <v>101</v>
       </c>
     </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A103" s="7">
+    <row r="104" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A104" s="6">
         <f t="shared" si="1"/>
         <v>102</v>
       </c>
     </row>
-    <row r="104" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A104" s="7">
+    <row r="105" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A105" s="6">
         <f t="shared" si="1"/>
         <v>103</v>
       </c>
     </row>
-    <row r="105" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A105" s="7">
+    <row r="106" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A106" s="6">
         <f t="shared" si="1"/>
         <v>104</v>
       </c>
     </row>
-    <row r="106" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A106" s="7">
+    <row r="107" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A107" s="6">
         <f t="shared" si="1"/>
         <v>105</v>
       </c>
     </row>
-    <row r="107" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A107" s="7">
+    <row r="108" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A108" s="6">
         <f t="shared" si="1"/>
         <v>106</v>
       </c>
     </row>
-    <row r="108" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A108" s="7">
+    <row r="109" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A109" s="6">
         <f t="shared" si="1"/>
         <v>107</v>
       </c>
     </row>
-    <row r="109" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A109" s="7">
+    <row r="110" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A110" s="6">
         <f t="shared" si="1"/>
         <v>108</v>
       </c>
     </row>
-    <row r="110" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A110" s="7">
+    <row r="111" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A111" s="6">
         <f t="shared" si="1"/>
         <v>109</v>
       </c>
     </row>
-    <row r="111" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A111" s="7">
+    <row r="112" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A112" s="6">
         <f t="shared" si="1"/>
         <v>110</v>
       </c>
     </row>
-    <row r="112" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A112" s="7">
+    <row r="113" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A113" s="6">
         <f t="shared" si="1"/>
         <v>111</v>
       </c>
     </row>
-    <row r="113" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A113" s="7">
+    <row r="114" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A114" s="6">
         <f t="shared" si="1"/>
         <v>112</v>
       </c>
     </row>
-    <row r="114" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A114" s="7">
+    <row r="115" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A115" s="6">
         <f t="shared" si="1"/>
         <v>113</v>
       </c>
     </row>
-    <row r="115" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A115" s="7">
+    <row r="116" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A116" s="6">
         <f t="shared" si="1"/>
         <v>114</v>
       </c>
     </row>
-    <row r="116" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A116" s="7">
+    <row r="117" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A117" s="6">
         <f t="shared" si="1"/>
         <v>115</v>
       </c>
     </row>
-    <row r="117" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A117" s="7">
+    <row r="118" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A118" s="6">
         <f t="shared" si="1"/>
         <v>116</v>
       </c>
     </row>
-    <row r="118" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A118" s="7">
+    <row r="119" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A119" s="6">
         <f t="shared" si="1"/>
         <v>117</v>
       </c>
     </row>
-    <row r="119" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A119" s="7">
+    <row r="120" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A120" s="6">
         <f t="shared" si="1"/>
         <v>118</v>
       </c>
     </row>
-    <row r="120" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A120" s="7">
+    <row r="121" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A121" s="6">
         <f t="shared" si="1"/>
         <v>119</v>
       </c>
     </row>
-    <row r="121" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A121" s="7">
+    <row r="122" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A122" s="6">
         <f t="shared" si="1"/>
         <v>120</v>
       </c>
     </row>
-    <row r="122" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A122" s="7">
+    <row r="123" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A123" s="6">
         <f t="shared" si="1"/>
         <v>121</v>
       </c>
     </row>
-    <row r="123" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A123" s="7">
+    <row r="124" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A124" s="6">
         <f t="shared" si="1"/>
         <v>122</v>
       </c>
     </row>
-    <row r="124" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A124" s="7">
+    <row r="125" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A125" s="6">
         <f t="shared" si="1"/>
         <v>123</v>
       </c>
     </row>
-    <row r="125" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A125" s="7">
+    <row r="126" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A126" s="6">
         <f t="shared" si="1"/>
         <v>124</v>
       </c>
     </row>
-    <row r="126" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A126" s="7">
+    <row r="127" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A127" s="6">
         <f t="shared" si="1"/>
         <v>125</v>
       </c>
     </row>
-    <row r="127" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A127" s="7">
+    <row r="128" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A128" s="6">
         <f t="shared" si="1"/>
         <v>126</v>
       </c>
     </row>
-    <row r="128" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A128" s="7">
+    <row r="129" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A129" s="6">
         <f t="shared" si="1"/>
         <v>127</v>
       </c>
     </row>
-    <row r="129" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A129" s="7">
+    <row r="130" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A130" s="6">
         <f t="shared" si="1"/>
         <v>128</v>
       </c>
     </row>
-    <row r="130" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A130" s="7">
+    <row r="131" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A131" s="6">
         <f t="shared" si="1"/>
         <v>129</v>
       </c>
     </row>
-    <row r="131" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A131" s="7">
+    <row r="132" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A132" s="6">
         <f t="shared" si="1"/>
         <v>130</v>
       </c>
     </row>
-    <row r="132" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A132" s="7">
+    <row r="133" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A133" s="6">
         <f t="shared" si="1"/>
         <v>131</v>
       </c>
     </row>
-    <row r="133" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A133" s="7">
+    <row r="134" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A134" s="6">
         <f t="shared" si="1"/>
         <v>132</v>
       </c>
     </row>
-    <row r="134" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A134" s="7">
+    <row r="135" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A135" s="6">
         <f t="shared" si="1"/>
         <v>133</v>
       </c>
     </row>
-    <row r="135" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A135" s="7">
+    <row r="136" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A136" s="6">
         <f t="shared" si="1"/>
         <v>134</v>
       </c>
     </row>
-    <row r="136" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A136" s="7">
+    <row r="137" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A137" s="6">
         <f t="shared" si="1"/>
         <v>135</v>
       </c>
     </row>
-    <row r="137" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A137" s="7">
+    <row r="138" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A138" s="6">
         <f t="shared" si="1"/>
         <v>136</v>
       </c>
     </row>
-    <row r="138" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A138" s="7">
-        <f t="shared" ref="A138:A201" si="2">SUM(A137+1)</f>
+    <row r="139" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A139" s="6">
+        <f t="shared" si="1"/>
         <v>137</v>
       </c>
     </row>
-    <row r="139" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A139" s="7">
-        <f t="shared" si="2"/>
+    <row r="140" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A140" s="6">
+        <f t="shared" ref="A140:A203" si="2">SUM(A139+1)</f>
         <v>138</v>
       </c>
     </row>
-    <row r="140" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A140" s="7">
+    <row r="141" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A141" s="6">
         <f t="shared" si="2"/>
         <v>139</v>
       </c>
     </row>
-    <row r="141" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A141" s="7">
+    <row r="142" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A142" s="6">
         <f t="shared" si="2"/>
         <v>140</v>
       </c>
     </row>
-    <row r="142" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A142" s="7">
+    <row r="143" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A143" s="6">
         <f t="shared" si="2"/>
         <v>141</v>
       </c>
     </row>
-    <row r="143" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A143" s="7">
+    <row r="144" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A144" s="6">
         <f t="shared" si="2"/>
         <v>142</v>
       </c>
     </row>
-    <row r="144" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A144" s="7">
+    <row r="145" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A145" s="6">
         <f t="shared" si="2"/>
         <v>143</v>
       </c>
     </row>
-    <row r="145" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A145" s="7">
+    <row r="146" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A146" s="6">
         <f t="shared" si="2"/>
         <v>144</v>
       </c>
     </row>
-    <row r="146" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A146" s="7">
+    <row r="147" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A147" s="6">
         <f t="shared" si="2"/>
         <v>145</v>
       </c>
     </row>
-    <row r="147" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A147" s="7">
+    <row r="148" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A148" s="6">
         <f t="shared" si="2"/>
         <v>146</v>
       </c>
     </row>
-    <row r="148" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A148" s="7">
+    <row r="149" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A149" s="6">
         <f t="shared" si="2"/>
         <v>147</v>
       </c>
     </row>
-    <row r="149" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A149" s="7">
+    <row r="150" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A150" s="6">
         <f t="shared" si="2"/>
         <v>148</v>
       </c>
     </row>
-    <row r="150" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A150" s="7">
+    <row r="151" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A151" s="6">
         <f t="shared" si="2"/>
         <v>149</v>
       </c>
     </row>
-    <row r="151" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A151" s="7">
+    <row r="152" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A152" s="6">
         <f t="shared" si="2"/>
         <v>150</v>
       </c>
     </row>
-    <row r="152" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A152" s="7">
+    <row r="153" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A153" s="6">
         <f t="shared" si="2"/>
         <v>151</v>
       </c>
     </row>
-    <row r="153" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A153" s="7">
+    <row r="154" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A154" s="6">
         <f t="shared" si="2"/>
         <v>152</v>
       </c>
     </row>
-    <row r="154" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A154" s="7">
+    <row r="155" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A155" s="6">
         <f t="shared" si="2"/>
         <v>153</v>
       </c>
     </row>
-    <row r="155" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A155" s="7">
+    <row r="156" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A156" s="6">
         <f t="shared" si="2"/>
         <v>154</v>
       </c>
     </row>
-    <row r="156" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A156" s="7">
+    <row r="157" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A157" s="6">
         <f t="shared" si="2"/>
         <v>155</v>
       </c>
     </row>
-    <row r="157" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A157" s="7">
+    <row r="158" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A158" s="6">
         <f t="shared" si="2"/>
         <v>156</v>
       </c>
     </row>
-    <row r="158" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A158" s="7">
+    <row r="159" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A159" s="6">
         <f t="shared" si="2"/>
         <v>157</v>
       </c>
     </row>
-    <row r="159" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A159" s="7">
+    <row r="160" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A160" s="6">
         <f t="shared" si="2"/>
         <v>158</v>
       </c>
     </row>
-    <row r="160" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A160" s="7">
+    <row r="161" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A161" s="6">
         <f t="shared" si="2"/>
         <v>159</v>
       </c>
     </row>
-    <row r="161" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A161" s="7">
+    <row r="162" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A162" s="6">
         <f t="shared" si="2"/>
         <v>160</v>
       </c>
     </row>
-    <row r="162" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A162" s="7">
+    <row r="163" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A163" s="6">
         <f t="shared" si="2"/>
         <v>161</v>
       </c>
     </row>
-    <row r="163" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A163" s="7">
+    <row r="164" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A164" s="6">
         <f t="shared" si="2"/>
         <v>162</v>
       </c>
     </row>
-    <row r="164" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A164" s="7">
+    <row r="165" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A165" s="6">
         <f t="shared" si="2"/>
         <v>163</v>
       </c>
     </row>
-    <row r="165" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A165" s="7">
+    <row r="166" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A166" s="6">
         <f t="shared" si="2"/>
         <v>164</v>
       </c>
     </row>
-    <row r="166" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A166" s="7">
+    <row r="167" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A167" s="6">
         <f t="shared" si="2"/>
         <v>165</v>
       </c>
     </row>
-    <row r="167" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A167" s="7">
+    <row r="168" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A168" s="6">
         <f t="shared" si="2"/>
         <v>166</v>
       </c>
     </row>
-    <row r="168" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A168" s="7">
+    <row r="169" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A169" s="6">
         <f t="shared" si="2"/>
         <v>167</v>
       </c>
     </row>
-    <row r="169" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A169" s="7">
+    <row r="170" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A170" s="6">
         <f t="shared" si="2"/>
         <v>168</v>
       </c>
     </row>
-    <row r="170" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A170" s="7">
+    <row r="171" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A171" s="6">
         <f t="shared" si="2"/>
         <v>169</v>
       </c>
     </row>
-    <row r="171" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A171" s="7">
+    <row r="172" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A172" s="6">
         <f t="shared" si="2"/>
         <v>170</v>
       </c>
     </row>
-    <row r="172" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A172" s="7">
+    <row r="173" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A173" s="6">
         <f t="shared" si="2"/>
         <v>171</v>
       </c>
     </row>
-    <row r="173" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A173" s="7">
+    <row r="174" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A174" s="6">
         <f t="shared" si="2"/>
         <v>172</v>
       </c>
     </row>
-    <row r="174" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A174" s="7">
+    <row r="175" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A175" s="6">
         <f t="shared" si="2"/>
         <v>173</v>
       </c>
     </row>
-    <row r="175" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A175" s="7">
+    <row r="176" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A176" s="6">
         <f t="shared" si="2"/>
         <v>174</v>
       </c>
     </row>
-    <row r="176" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A176" s="7">
+    <row r="177" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A177" s="6">
         <f t="shared" si="2"/>
         <v>175</v>
       </c>
     </row>
-    <row r="177" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A177" s="7">
+    <row r="178" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A178" s="6">
         <f t="shared" si="2"/>
         <v>176</v>
       </c>
     </row>
-    <row r="178" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A178" s="7">
+    <row r="179" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A179" s="6">
         <f t="shared" si="2"/>
         <v>177</v>
       </c>
     </row>
-    <row r="179" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A179" s="7">
+    <row r="180" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A180" s="6">
         <f t="shared" si="2"/>
         <v>178</v>
       </c>
     </row>
-    <row r="180" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A180" s="7">
+    <row r="181" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A181" s="6">
         <f t="shared" si="2"/>
         <v>179</v>
       </c>
     </row>
-    <row r="181" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A181" s="7">
+    <row r="182" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A182" s="6">
         <f t="shared" si="2"/>
         <v>180</v>
       </c>
     </row>
-    <row r="182" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A182" s="7">
+    <row r="183" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A183" s="6">
         <f t="shared" si="2"/>
         <v>181</v>
       </c>
     </row>
-    <row r="183" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A183" s="7">
+    <row r="184" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A184" s="6">
         <f t="shared" si="2"/>
         <v>182</v>
       </c>
     </row>
-    <row r="184" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A184" s="7">
+    <row r="185" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A185" s="6">
         <f t="shared" si="2"/>
         <v>183</v>
       </c>
     </row>
-    <row r="185" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A185" s="7">
+    <row r="186" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A186" s="6">
         <f t="shared" si="2"/>
         <v>184</v>
       </c>
     </row>
-    <row r="186" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A186" s="7">
+    <row r="187" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A187" s="6">
         <f t="shared" si="2"/>
         <v>185</v>
       </c>
     </row>
-    <row r="187" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A187" s="7">
+    <row r="188" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A188" s="6">
         <f t="shared" si="2"/>
         <v>186</v>
       </c>
     </row>
-    <row r="188" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A188" s="7">
+    <row r="189" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A189" s="6">
         <f t="shared" si="2"/>
         <v>187</v>
       </c>
     </row>
-    <row r="189" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A189" s="7">
+    <row r="190" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A190" s="6">
         <f t="shared" si="2"/>
         <v>188</v>
       </c>
     </row>
-    <row r="190" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A190" s="7">
+    <row r="191" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A191" s="6">
         <f t="shared" si="2"/>
         <v>189</v>
       </c>
     </row>
-    <row r="191" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A191" s="7">
+    <row r="192" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A192" s="6">
         <f t="shared" si="2"/>
         <v>190</v>
       </c>
     </row>
-    <row r="192" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A192" s="7">
+    <row r="193" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A193" s="6">
         <f t="shared" si="2"/>
         <v>191</v>
       </c>
     </row>
-    <row r="193" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A193" s="7">
+    <row r="194" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A194" s="6">
         <f t="shared" si="2"/>
         <v>192</v>
       </c>
     </row>
-    <row r="194" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A194" s="7">
+    <row r="195" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A195" s="6">
         <f t="shared" si="2"/>
         <v>193</v>
       </c>
     </row>
-    <row r="195" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A195" s="7">
+    <row r="196" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A196" s="6">
         <f t="shared" si="2"/>
         <v>194</v>
       </c>
     </row>
-    <row r="196" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A196" s="7">
+    <row r="197" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A197" s="6">
         <f t="shared" si="2"/>
         <v>195</v>
       </c>
     </row>
-    <row r="197" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A197" s="7">
+    <row r="198" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A198" s="6">
         <f t="shared" si="2"/>
         <v>196</v>
       </c>
     </row>
-    <row r="198" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A198" s="7">
+    <row r="199" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A199" s="6">
         <f t="shared" si="2"/>
         <v>197</v>
       </c>
     </row>
-    <row r="199" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A199" s="7">
+    <row r="200" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A200" s="6">
         <f t="shared" si="2"/>
         <v>198</v>
       </c>
     </row>
-    <row r="200" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A200" s="7">
+    <row r="201" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A201" s="6">
         <f t="shared" si="2"/>
         <v>199</v>
       </c>
     </row>
-    <row r="201" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A201" s="7">
+    <row r="202" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A202" s="6">
         <f t="shared" si="2"/>
         <v>200</v>
       </c>
     </row>
-    <row r="202" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A202" s="7">
-        <f t="shared" ref="A202:A265" si="3">SUM(A201+1)</f>
+    <row r="203" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A203" s="6">
+        <f t="shared" si="2"/>
         <v>201</v>
       </c>
     </row>
-    <row r="203" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A203" s="7">
-        <f t="shared" si="3"/>
+    <row r="204" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A204" s="6">
+        <f t="shared" ref="A204:A267" si="3">SUM(A203+1)</f>
         <v>202</v>
       </c>
     </row>
-    <row r="204" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A204" s="7">
+    <row r="205" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A205" s="6">
         <f t="shared" si="3"/>
         <v>203</v>
       </c>
     </row>
-    <row r="205" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A205" s="7">
+    <row r="206" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A206" s="6">
         <f t="shared" si="3"/>
         <v>204</v>
       </c>
     </row>
-    <row r="206" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A206" s="7">
+    <row r="207" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A207" s="6">
         <f t="shared" si="3"/>
         <v>205</v>
       </c>
     </row>
-    <row r="207" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A207" s="7">
+    <row r="208" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A208" s="6">
         <f t="shared" si="3"/>
         <v>206</v>
       </c>
     </row>
-    <row r="208" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A208" s="7">
+    <row r="209" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A209" s="6">
         <f t="shared" si="3"/>
         <v>207</v>
       </c>
     </row>
-    <row r="209" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A209" s="7">
+    <row r="210" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A210" s="6">
         <f t="shared" si="3"/>
         <v>208</v>
       </c>
     </row>
-    <row r="210" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A210" s="7">
+    <row r="211" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A211" s="6">
         <f t="shared" si="3"/>
         <v>209</v>
       </c>
     </row>
-    <row r="211" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A211" s="7">
+    <row r="212" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A212" s="6">
         <f t="shared" si="3"/>
         <v>210</v>
       </c>
     </row>
-    <row r="212" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A212" s="7">
+    <row r="213" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A213" s="6">
         <f t="shared" si="3"/>
         <v>211</v>
       </c>
     </row>
-    <row r="213" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A213" s="7">
+    <row r="214" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A214" s="6">
         <f t="shared" si="3"/>
         <v>212</v>
       </c>
     </row>
-    <row r="214" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A214" s="7">
+    <row r="215" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A215" s="6">
         <f t="shared" si="3"/>
         <v>213</v>
       </c>
     </row>
-    <row r="215" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A215" s="7">
+    <row r="216" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A216" s="6">
         <f t="shared" si="3"/>
         <v>214</v>
       </c>
     </row>
-    <row r="216" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A216" s="7">
+    <row r="217" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A217" s="6">
         <f t="shared" si="3"/>
         <v>215</v>
       </c>
     </row>
-    <row r="217" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A217" s="7">
+    <row r="218" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A218" s="6">
         <f t="shared" si="3"/>
         <v>216</v>
       </c>
     </row>
-    <row r="218" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A218" s="7">
+    <row r="219" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A219" s="6">
         <f t="shared" si="3"/>
         <v>217</v>
       </c>
     </row>
-    <row r="219" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A219" s="7">
+    <row r="220" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A220" s="6">
         <f t="shared" si="3"/>
         <v>218</v>
       </c>
     </row>
-    <row r="220" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A220" s="7">
+    <row r="221" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A221" s="6">
         <f t="shared" si="3"/>
         <v>219</v>
       </c>
     </row>
-    <row r="221" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A221" s="7">
+    <row r="222" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A222" s="6">
         <f t="shared" si="3"/>
         <v>220</v>
       </c>
     </row>
-    <row r="222" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A222" s="7">
+    <row r="223" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A223" s="6">
         <f t="shared" si="3"/>
         <v>221</v>
       </c>
     </row>
-    <row r="223" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A223" s="7">
+    <row r="224" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A224" s="6">
         <f t="shared" si="3"/>
         <v>222</v>
       </c>
     </row>
-    <row r="224" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A224" s="7">
+    <row r="225" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A225" s="6">
         <f t="shared" si="3"/>
         <v>223</v>
       </c>
     </row>
-    <row r="225" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A225" s="7">
+    <row r="226" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A226" s="6">
         <f t="shared" si="3"/>
         <v>224</v>
       </c>
     </row>
-    <row r="226" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A226" s="7">
+    <row r="227" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A227" s="6">
         <f t="shared" si="3"/>
         <v>225</v>
       </c>
     </row>
-    <row r="227" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A227" s="7">
+    <row r="228" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A228" s="6">
         <f t="shared" si="3"/>
         <v>226</v>
       </c>
     </row>
-    <row r="228" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A228" s="7">
+    <row r="229" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A229" s="6">
         <f t="shared" si="3"/>
         <v>227</v>
       </c>
     </row>
-    <row r="229" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A229" s="7">
+    <row r="230" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A230" s="6">
         <f t="shared" si="3"/>
         <v>228</v>
       </c>
     </row>
-    <row r="230" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A230" s="7">
+    <row r="231" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A231" s="6">
         <f t="shared" si="3"/>
         <v>229</v>
       </c>
     </row>
-    <row r="231" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A231" s="7">
+    <row r="232" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A232" s="6">
         <f t="shared" si="3"/>
         <v>230</v>
       </c>
     </row>
-    <row r="232" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A232" s="7">
+    <row r="233" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A233" s="6">
         <f t="shared" si="3"/>
         <v>231</v>
       </c>
     </row>
-    <row r="233" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A233" s="7">
+    <row r="234" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A234" s="6">
         <f t="shared" si="3"/>
         <v>232</v>
       </c>
     </row>
-    <row r="234" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A234" s="7">
+    <row r="235" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A235" s="6">
         <f t="shared" si="3"/>
         <v>233</v>
       </c>
     </row>
-    <row r="235" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A235" s="7">
+    <row r="236" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A236" s="6">
         <f t="shared" si="3"/>
         <v>234</v>
       </c>
     </row>
-    <row r="236" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A236" s="7">
+    <row r="237" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A237" s="6">
         <f t="shared" si="3"/>
         <v>235</v>
       </c>
     </row>
-    <row r="237" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A237" s="7">
+    <row r="238" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A238" s="6">
         <f t="shared" si="3"/>
         <v>236</v>
       </c>
     </row>
-    <row r="238" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A238" s="7">
+    <row r="239" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A239" s="6">
         <f t="shared" si="3"/>
         <v>237</v>
       </c>
     </row>
-    <row r="239" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A239" s="7">
+    <row r="240" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A240" s="6">
         <f t="shared" si="3"/>
         <v>238</v>
       </c>
     </row>
-    <row r="240" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A240" s="7">
+    <row r="241" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A241" s="6">
         <f t="shared" si="3"/>
         <v>239</v>
       </c>
     </row>
-    <row r="241" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A241" s="7">
+    <row r="242" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A242" s="6">
         <f t="shared" si="3"/>
         <v>240</v>
       </c>
     </row>
-    <row r="242" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A242" s="7">
+    <row r="243" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A243" s="6">
         <f t="shared" si="3"/>
         <v>241</v>
       </c>
     </row>
-    <row r="243" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A243" s="7">
+    <row r="244" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A244" s="6">
         <f t="shared" si="3"/>
         <v>242</v>
       </c>
     </row>
-    <row r="244" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A244" s="7">
+    <row r="245" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A245" s="6">
         <f t="shared" si="3"/>
         <v>243</v>
       </c>
     </row>
-    <row r="245" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A245" s="7">
+    <row r="246" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A246" s="6">
         <f t="shared" si="3"/>
         <v>244</v>
       </c>
     </row>
-    <row r="246" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A246" s="7">
+    <row r="247" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A247" s="6">
         <f t="shared" si="3"/>
         <v>245</v>
       </c>
     </row>
-    <row r="247" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A247" s="7">
+    <row r="248" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A248" s="6">
         <f t="shared" si="3"/>
         <v>246</v>
       </c>
     </row>
-    <row r="248" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A248" s="7">
+    <row r="249" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A249" s="6">
         <f t="shared" si="3"/>
         <v>247</v>
       </c>
     </row>
-    <row r="249" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A249" s="7">
+    <row r="250" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A250" s="6">
         <f t="shared" si="3"/>
         <v>248</v>
       </c>
     </row>
-    <row r="250" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A250" s="7">
+    <row r="251" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A251" s="6">
         <f t="shared" si="3"/>
         <v>249</v>
       </c>
     </row>
-    <row r="251" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A251" s="7">
+    <row r="252" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A252" s="6">
         <f t="shared" si="3"/>
         <v>250</v>
       </c>
     </row>
-    <row r="252" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A252" s="7">
+    <row r="253" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A253" s="6">
         <f t="shared" si="3"/>
         <v>251</v>
       </c>
     </row>
-    <row r="253" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A253" s="7">
+    <row r="254" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A254" s="6">
         <f t="shared" si="3"/>
         <v>252</v>
       </c>
     </row>
-    <row r="254" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A254" s="7">
+    <row r="255" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A255" s="6">
         <f t="shared" si="3"/>
         <v>253</v>
       </c>
     </row>
-    <row r="255" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A255" s="7">
+    <row r="256" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A256" s="6">
         <f t="shared" si="3"/>
         <v>254</v>
       </c>
     </row>
-    <row r="256" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A256" s="7">
+    <row r="257" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A257" s="6">
         <f t="shared" si="3"/>
         <v>255</v>
       </c>
     </row>
-    <row r="257" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A257" s="7">
+    <row r="258" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A258" s="6">
         <f t="shared" si="3"/>
         <v>256</v>
       </c>
     </row>
-    <row r="258" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A258" s="7">
+    <row r="259" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A259" s="6">
         <f t="shared" si="3"/>
         <v>257</v>
       </c>
     </row>
-    <row r="259" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A259" s="7">
+    <row r="260" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A260" s="6">
         <f t="shared" si="3"/>
         <v>258</v>
       </c>
     </row>
-    <row r="260" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A260" s="7">
+    <row r="261" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A261" s="6">
         <f t="shared" si="3"/>
         <v>259</v>
       </c>
     </row>
-    <row r="261" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A261" s="7">
+    <row r="262" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A262" s="6">
         <f t="shared" si="3"/>
         <v>260</v>
       </c>
     </row>
-    <row r="262" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A262" s="7">
+    <row r="263" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A263" s="6">
         <f t="shared" si="3"/>
         <v>261</v>
       </c>
     </row>
-    <row r="263" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A263" s="7">
+    <row r="264" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A264" s="6">
         <f t="shared" si="3"/>
         <v>262</v>
       </c>
     </row>
-    <row r="264" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A264" s="7">
+    <row r="265" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A265" s="6">
         <f t="shared" si="3"/>
         <v>263</v>
       </c>
     </row>
-    <row r="265" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A265" s="7">
+    <row r="266" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A266" s="6">
         <f t="shared" si="3"/>
         <v>264</v>
       </c>
     </row>
-    <row r="266" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A266" s="7">
-        <f t="shared" ref="A266:A329" si="4">SUM(A265+1)</f>
+    <row r="267" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A267" s="6">
+        <f t="shared" si="3"/>
         <v>265</v>
       </c>
     </row>
-    <row r="267" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A267" s="7">
-        <f t="shared" si="4"/>
+    <row r="268" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A268" s="6">
+        <f t="shared" ref="A268:A331" si="4">SUM(A267+1)</f>
         <v>266</v>
       </c>
     </row>
-    <row r="268" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A268" s="7">
+    <row r="269" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A269" s="6">
         <f t="shared" si="4"/>
         <v>267</v>
       </c>
     </row>
-    <row r="269" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A269" s="7">
+    <row r="270" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A270" s="6">
         <f t="shared" si="4"/>
         <v>268</v>
       </c>
     </row>
-    <row r="270" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A270" s="7">
+    <row r="271" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A271" s="6">
         <f t="shared" si="4"/>
         <v>269</v>
       </c>
     </row>
-    <row r="271" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A271" s="7">
+    <row r="272" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A272" s="6">
         <f t="shared" si="4"/>
         <v>270</v>
       </c>
     </row>
-    <row r="272" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A272" s="7">
+    <row r="273" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A273" s="6">
         <f t="shared" si="4"/>
         <v>271</v>
       </c>
     </row>
-    <row r="273" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A273" s="7">
+    <row r="274" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A274" s="6">
         <f t="shared" si="4"/>
         <v>272</v>
       </c>
     </row>
-    <row r="274" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A274" s="7">
+    <row r="275" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A275" s="6">
         <f t="shared" si="4"/>
         <v>273</v>
       </c>
     </row>
-    <row r="275" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A275" s="7">
+    <row r="276" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A276" s="6">
         <f t="shared" si="4"/>
         <v>274</v>
       </c>
     </row>
-    <row r="276" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A276" s="7">
+    <row r="277" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A277" s="6">
         <f t="shared" si="4"/>
         <v>275</v>
       </c>
     </row>
-    <row r="277" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A277" s="7">
+    <row r="278" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A278" s="6">
         <f t="shared" si="4"/>
         <v>276</v>
       </c>
     </row>
-    <row r="278" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A278" s="7">
+    <row r="279" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A279" s="6">
         <f t="shared" si="4"/>
         <v>277</v>
       </c>
     </row>
-    <row r="279" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A279" s="7">
+    <row r="280" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A280" s="6">
         <f t="shared" si="4"/>
         <v>278</v>
       </c>
     </row>
-    <row r="280" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A280" s="7">
+    <row r="281" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A281" s="6">
         <f t="shared" si="4"/>
         <v>279</v>
       </c>
     </row>
-    <row r="281" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A281" s="7">
+    <row r="282" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A282" s="6">
         <f t="shared" si="4"/>
         <v>280</v>
       </c>
     </row>
-    <row r="282" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A282" s="7">
+    <row r="283" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A283" s="6">
         <f t="shared" si="4"/>
         <v>281</v>
       </c>
     </row>
-    <row r="283" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A283" s="7">
+    <row r="284" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A284" s="6">
         <f t="shared" si="4"/>
         <v>282</v>
       </c>
     </row>
-    <row r="284" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A284" s="7">
+    <row r="285" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A285" s="6">
         <f t="shared" si="4"/>
         <v>283</v>
       </c>
     </row>
-    <row r="285" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A285" s="7">
+    <row r="286" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A286" s="6">
         <f t="shared" si="4"/>
         <v>284</v>
       </c>
     </row>
-    <row r="286" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A286" s="7">
+    <row r="287" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A287" s="6">
         <f t="shared" si="4"/>
         <v>285</v>
       </c>
     </row>
-    <row r="287" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A287" s="7">
+    <row r="288" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A288" s="6">
         <f t="shared" si="4"/>
         <v>286</v>
       </c>
     </row>
-    <row r="288" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A288" s="7">
+    <row r="289" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A289" s="6">
         <f t="shared" si="4"/>
         <v>287</v>
       </c>
     </row>
-    <row r="289" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A289" s="7">
+    <row r="290" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A290" s="6">
         <f t="shared" si="4"/>
         <v>288</v>
       </c>
     </row>
-    <row r="290" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A290" s="7">
+    <row r="291" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A291" s="6">
         <f t="shared" si="4"/>
         <v>289</v>
       </c>
     </row>
-    <row r="291" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A291" s="7">
+    <row r="292" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A292" s="6">
         <f t="shared" si="4"/>
         <v>290</v>
       </c>
     </row>
-    <row r="292" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A292" s="7">
+    <row r="293" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A293" s="6">
         <f t="shared" si="4"/>
         <v>291</v>
       </c>
     </row>
-    <row r="293" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A293" s="7">
+    <row r="294" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A294" s="6">
         <f t="shared" si="4"/>
         <v>292</v>
       </c>
     </row>
-    <row r="294" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A294" s="7">
+    <row r="295" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A295" s="6">
         <f t="shared" si="4"/>
         <v>293</v>
       </c>
     </row>
-    <row r="295" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A295" s="7">
+    <row r="296" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A296" s="6">
         <f t="shared" si="4"/>
         <v>294</v>
       </c>
     </row>
-    <row r="296" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A296" s="7">
+    <row r="297" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A297" s="6">
         <f t="shared" si="4"/>
         <v>295</v>
       </c>
     </row>
-    <row r="297" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A297" s="7">
+    <row r="298" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A298" s="6">
         <f t="shared" si="4"/>
         <v>296</v>
       </c>
     </row>
-    <row r="298" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A298" s="7">
+    <row r="299" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A299" s="6">
         <f t="shared" si="4"/>
         <v>297</v>
       </c>
     </row>
-    <row r="299" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A299" s="7">
+    <row r="300" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A300" s="6">
         <f t="shared" si="4"/>
         <v>298</v>
       </c>
     </row>
-    <row r="300" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A300" s="7">
+    <row r="301" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A301" s="6">
         <f t="shared" si="4"/>
         <v>299</v>
       </c>
     </row>
-    <row r="301" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A301" s="7">
+    <row r="302" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A302" s="6">
         <f t="shared" si="4"/>
         <v>300</v>
       </c>
     </row>
-    <row r="302" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A302" s="7">
+    <row r="303" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A303" s="6">
         <f t="shared" si="4"/>
         <v>301</v>
       </c>
     </row>
-    <row r="303" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A303" s="7">
+    <row r="304" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A304" s="6">
         <f t="shared" si="4"/>
         <v>302</v>
       </c>
     </row>
-    <row r="304" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A304" s="7">
+    <row r="305" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A305" s="6">
         <f t="shared" si="4"/>
         <v>303</v>
       </c>
     </row>
-    <row r="305" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A305" s="7">
+    <row r="306" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A306" s="6">
         <f t="shared" si="4"/>
         <v>304</v>
       </c>
     </row>
-    <row r="306" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A306" s="7">
+    <row r="307" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A307" s="6">
         <f t="shared" si="4"/>
         <v>305</v>
       </c>
     </row>
-    <row r="307" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A307" s="7">
+    <row r="308" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A308" s="6">
         <f t="shared" si="4"/>
         <v>306</v>
       </c>
     </row>
-    <row r="308" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A308" s="7">
+    <row r="309" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A309" s="6">
         <f t="shared" si="4"/>
         <v>307</v>
       </c>
     </row>
-    <row r="309" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A309" s="7">
+    <row r="310" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A310" s="6">
         <f t="shared" si="4"/>
         <v>308</v>
       </c>
     </row>
-    <row r="310" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A310" s="7">
+    <row r="311" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A311" s="6">
         <f t="shared" si="4"/>
         <v>309</v>
       </c>
     </row>
-    <row r="311" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A311" s="7">
+    <row r="312" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A312" s="6">
         <f t="shared" si="4"/>
         <v>310</v>
       </c>
     </row>
-    <row r="312" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A312" s="7">
+    <row r="313" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A313" s="6">
         <f t="shared" si="4"/>
         <v>311</v>
       </c>
     </row>
-    <row r="313" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A313" s="7">
+    <row r="314" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A314" s="6">
         <f t="shared" si="4"/>
         <v>312</v>
       </c>
     </row>
-    <row r="314" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A314" s="7">
+    <row r="315" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A315" s="6">
         <f t="shared" si="4"/>
         <v>313</v>
       </c>
     </row>
-    <row r="315" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A315" s="7">
+    <row r="316" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A316" s="6">
         <f t="shared" si="4"/>
         <v>314</v>
       </c>
     </row>
-    <row r="316" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A316" s="7">
+    <row r="317" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A317" s="6">
         <f t="shared" si="4"/>
         <v>315</v>
       </c>
     </row>
-    <row r="317" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A317" s="7">
+    <row r="318" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A318" s="6">
         <f t="shared" si="4"/>
         <v>316</v>
       </c>
     </row>
-    <row r="318" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A318" s="7">
+    <row r="319" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A319" s="6">
         <f t="shared" si="4"/>
         <v>317</v>
       </c>
     </row>
-    <row r="319" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A319" s="7">
+    <row r="320" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A320" s="6">
         <f t="shared" si="4"/>
         <v>318</v>
       </c>
     </row>
-    <row r="320" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A320" s="7">
+    <row r="321" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A321" s="6">
         <f t="shared" si="4"/>
         <v>319</v>
       </c>
     </row>
-    <row r="321" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A321" s="7">
+    <row r="322" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A322" s="6">
         <f t="shared" si="4"/>
         <v>320</v>
       </c>
     </row>
-    <row r="322" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A322" s="7">
+    <row r="323" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A323" s="6">
         <f t="shared" si="4"/>
         <v>321</v>
       </c>
     </row>
-    <row r="323" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A323" s="7">
+    <row r="324" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A324" s="6">
         <f t="shared" si="4"/>
         <v>322</v>
       </c>
     </row>
-    <row r="324" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A324" s="7">
+    <row r="325" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A325" s="6">
         <f t="shared" si="4"/>
         <v>323</v>
       </c>
     </row>
-    <row r="325" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A325" s="7">
+    <row r="326" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A326" s="6">
         <f t="shared" si="4"/>
         <v>324</v>
       </c>
     </row>
-    <row r="326" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A326" s="7">
+    <row r="327" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A327" s="6">
         <f t="shared" si="4"/>
         <v>325</v>
       </c>
     </row>
-    <row r="327" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A327" s="7">
+    <row r="328" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A328" s="6">
         <f t="shared" si="4"/>
         <v>326</v>
       </c>
     </row>
-    <row r="328" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A328" s="7">
+    <row r="329" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A329" s="6">
         <f t="shared" si="4"/>
         <v>327</v>
       </c>
     </row>
-    <row r="329" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A329" s="7">
+    <row r="330" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A330" s="6">
         <f t="shared" si="4"/>
         <v>328</v>
       </c>
     </row>
-    <row r="330" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A330" s="7">
-        <f t="shared" ref="A330:A393" si="5">SUM(A329+1)</f>
+    <row r="331" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A331" s="6">
+        <f t="shared" si="4"/>
         <v>329</v>
       </c>
     </row>
-    <row r="331" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A331" s="7">
-        <f t="shared" si="5"/>
+    <row r="332" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A332" s="6">
+        <f t="shared" ref="A332:A395" si="5">SUM(A331+1)</f>
         <v>330</v>
       </c>
     </row>
-    <row r="332" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A332" s="7">
+    <row r="333" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A333" s="6">
         <f t="shared" si="5"/>
         <v>331</v>
       </c>
     </row>
-    <row r="333" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A333" s="7">
+    <row r="334" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A334" s="6">
         <f t="shared" si="5"/>
         <v>332</v>
       </c>
     </row>
-    <row r="334" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A334" s="7">
+    <row r="335" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A335" s="6">
         <f t="shared" si="5"/>
         <v>333</v>
       </c>
     </row>
-    <row r="335" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A335" s="7">
+    <row r="336" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A336" s="6">
         <f t="shared" si="5"/>
         <v>334</v>
       </c>
     </row>
-    <row r="336" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A336" s="7">
+    <row r="337" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A337" s="6">
         <f t="shared" si="5"/>
         <v>335</v>
       </c>
     </row>
-    <row r="337" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A337" s="7">
+    <row r="338" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A338" s="6">
         <f t="shared" si="5"/>
         <v>336</v>
       </c>
     </row>
-    <row r="338" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A338" s="7">
+    <row r="339" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A339" s="6">
         <f t="shared" si="5"/>
         <v>337</v>
       </c>
     </row>
-    <row r="339" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A339" s="7">
+    <row r="340" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A340" s="6">
         <f t="shared" si="5"/>
         <v>338</v>
       </c>
     </row>
-    <row r="340" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A340" s="7">
+    <row r="341" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A341" s="6">
         <f t="shared" si="5"/>
         <v>339</v>
       </c>
     </row>
-    <row r="341" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A341" s="7">
+    <row r="342" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A342" s="6">
         <f t="shared" si="5"/>
         <v>340</v>
       </c>
     </row>
-    <row r="342" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A342" s="7">
+    <row r="343" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A343" s="6">
         <f t="shared" si="5"/>
         <v>341</v>
       </c>
     </row>
-    <row r="343" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A343" s="7">
+    <row r="344" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A344" s="6">
         <f t="shared" si="5"/>
         <v>342</v>
       </c>
     </row>
-    <row r="344" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A344" s="7">
+    <row r="345" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A345" s="6">
         <f t="shared" si="5"/>
         <v>343</v>
       </c>
     </row>
-    <row r="345" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A345" s="7">
+    <row r="346" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A346" s="6">
         <f t="shared" si="5"/>
         <v>344</v>
       </c>
     </row>
-    <row r="346" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A346" s="7">
+    <row r="347" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A347" s="6">
         <f t="shared" si="5"/>
         <v>345</v>
       </c>
     </row>
-    <row r="347" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A347" s="7">
+    <row r="348" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A348" s="6">
         <f t="shared" si="5"/>
         <v>346</v>
       </c>
     </row>
-    <row r="348" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A348" s="7">
+    <row r="349" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A349" s="6">
         <f t="shared" si="5"/>
         <v>347</v>
       </c>
     </row>
-    <row r="349" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A349" s="7">
+    <row r="350" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A350" s="6">
         <f t="shared" si="5"/>
         <v>348</v>
       </c>
     </row>
-    <row r="350" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A350" s="7">
+    <row r="351" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A351" s="6">
         <f t="shared" si="5"/>
         <v>349</v>
       </c>
     </row>
-    <row r="351" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A351" s="7">
+    <row r="352" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A352" s="6">
         <f t="shared" si="5"/>
         <v>350</v>
       </c>
     </row>
-    <row r="352" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A352" s="7">
+    <row r="353" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A353" s="6">
         <f t="shared" si="5"/>
         <v>351</v>
       </c>
     </row>
-    <row r="353" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A353" s="7">
+    <row r="354" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A354" s="6">
         <f t="shared" si="5"/>
         <v>352</v>
       </c>
     </row>
-    <row r="354" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A354" s="7">
+    <row r="355" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A355" s="6">
         <f t="shared" si="5"/>
         <v>353</v>
       </c>
     </row>
-    <row r="355" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A355" s="7">
+    <row r="356" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A356" s="6">
         <f t="shared" si="5"/>
         <v>354</v>
       </c>
     </row>
-    <row r="356" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A356" s="7">
+    <row r="357" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A357" s="6">
         <f t="shared" si="5"/>
         <v>355</v>
       </c>
     </row>
-    <row r="357" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A357" s="7">
+    <row r="358" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A358" s="6">
         <f t="shared" si="5"/>
         <v>356</v>
       </c>
     </row>
-    <row r="358" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A358" s="7">
+    <row r="359" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A359" s="6">
         <f t="shared" si="5"/>
         <v>357</v>
       </c>
     </row>
-    <row r="359" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A359" s="7">
+    <row r="360" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A360" s="6">
         <f t="shared" si="5"/>
         <v>358</v>
       </c>
     </row>
-    <row r="360" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A360" s="7">
+    <row r="361" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A361" s="6">
         <f t="shared" si="5"/>
         <v>359</v>
       </c>
     </row>
-    <row r="361" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A361" s="7">
+    <row r="362" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A362" s="6">
         <f t="shared" si="5"/>
         <v>360</v>
       </c>
     </row>
-    <row r="362" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A362" s="7">
+    <row r="363" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A363" s="6">
         <f t="shared" si="5"/>
         <v>361</v>
       </c>
     </row>
-    <row r="363" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A363" s="7">
+    <row r="364" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A364" s="6">
         <f t="shared" si="5"/>
         <v>362</v>
       </c>
     </row>
-    <row r="364" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A364" s="7">
+    <row r="365" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A365" s="6">
         <f t="shared" si="5"/>
         <v>363</v>
       </c>
     </row>
-    <row r="365" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A365" s="7">
+    <row r="366" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A366" s="6">
         <f t="shared" si="5"/>
         <v>364</v>
       </c>
     </row>
-    <row r="366" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A366" s="7">
+    <row r="367" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A367" s="6">
         <f t="shared" si="5"/>
         <v>365</v>
       </c>
     </row>
-    <row r="367" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A367" s="7">
+    <row r="368" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A368" s="6">
         <f t="shared" si="5"/>
         <v>366</v>
       </c>
     </row>
-    <row r="368" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A368" s="7">
+    <row r="369" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A369" s="6">
         <f t="shared" si="5"/>
         <v>367</v>
       </c>
     </row>
-    <row r="369" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A369" s="7">
+    <row r="370" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A370" s="6">
         <f t="shared" si="5"/>
         <v>368</v>
       </c>
     </row>
-    <row r="370" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A370" s="7">
+    <row r="371" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A371" s="6">
         <f t="shared" si="5"/>
         <v>369</v>
       </c>
     </row>
-    <row r="371" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A371" s="7">
+    <row r="372" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A372" s="6">
         <f t="shared" si="5"/>
         <v>370</v>
       </c>
     </row>
-    <row r="372" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A372" s="7">
+    <row r="373" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A373" s="6">
         <f t="shared" si="5"/>
         <v>371</v>
       </c>
     </row>
-    <row r="373" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A373" s="7">
+    <row r="374" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A374" s="6">
         <f t="shared" si="5"/>
         <v>372</v>
       </c>
     </row>
-    <row r="374" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A374" s="7">
+    <row r="375" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A375" s="6">
         <f t="shared" si="5"/>
         <v>373</v>
       </c>
     </row>
-    <row r="375" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A375" s="7">
+    <row r="376" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A376" s="6">
         <f t="shared" si="5"/>
         <v>374</v>
       </c>
     </row>
-    <row r="376" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A376" s="7">
+    <row r="377" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A377" s="6">
         <f t="shared" si="5"/>
         <v>375</v>
       </c>
     </row>
-    <row r="377" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A377" s="7">
+    <row r="378" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A378" s="6">
         <f t="shared" si="5"/>
         <v>376</v>
       </c>
     </row>
-    <row r="378" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A378" s="7">
+    <row r="379" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A379" s="6">
         <f t="shared" si="5"/>
         <v>377</v>
       </c>
     </row>
-    <row r="379" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A379" s="7">
+    <row r="380" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A380" s="6">
         <f t="shared" si="5"/>
         <v>378</v>
       </c>
     </row>
-    <row r="380" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A380" s="7">
+    <row r="381" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A381" s="6">
         <f t="shared" si="5"/>
         <v>379</v>
       </c>
     </row>
-    <row r="381" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A381" s="7">
+    <row r="382" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A382" s="6">
         <f t="shared" si="5"/>
         <v>380</v>
       </c>
     </row>
-    <row r="382" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A382" s="7">
+    <row r="383" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A383" s="6">
         <f t="shared" si="5"/>
         <v>381</v>
       </c>
     </row>
-    <row r="383" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A383" s="7">
+    <row r="384" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A384" s="6">
         <f t="shared" si="5"/>
         <v>382</v>
       </c>
     </row>
-    <row r="384" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A384" s="7">
+    <row r="385" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A385" s="6">
         <f t="shared" si="5"/>
         <v>383</v>
       </c>
     </row>
-    <row r="385" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A385" s="7">
+    <row r="386" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A386" s="6">
         <f t="shared" si="5"/>
         <v>384</v>
       </c>
     </row>
-    <row r="386" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A386" s="7">
+    <row r="387" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A387" s="6">
         <f t="shared" si="5"/>
         <v>385</v>
       </c>
     </row>
-    <row r="387" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A387" s="7">
+    <row r="388" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A388" s="6">
         <f t="shared" si="5"/>
         <v>386</v>
       </c>
     </row>
-    <row r="388" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A388" s="7">
+    <row r="389" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A389" s="6">
         <f t="shared" si="5"/>
         <v>387</v>
       </c>
     </row>
-    <row r="389" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A389" s="7">
+    <row r="390" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A390" s="6">
         <f t="shared" si="5"/>
         <v>388</v>
       </c>
     </row>
-    <row r="390" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A390" s="7">
+    <row r="391" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A391" s="6">
         <f t="shared" si="5"/>
         <v>389</v>
       </c>
     </row>
-    <row r="391" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A391" s="7">
+    <row r="392" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A392" s="6">
         <f t="shared" si="5"/>
         <v>390</v>
       </c>
     </row>
-    <row r="392" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A392" s="7">
+    <row r="393" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A393" s="6">
         <f t="shared" si="5"/>
         <v>391</v>
       </c>
     </row>
-    <row r="393" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A393" s="7">
+    <row r="394" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A394" s="6">
         <f t="shared" si="5"/>
         <v>392</v>
       </c>
     </row>
-    <row r="394" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A394" s="7">
-        <f t="shared" ref="A394:A452" si="6">SUM(A393+1)</f>
+    <row r="395" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A395" s="6">
+        <f t="shared" si="5"/>
         <v>393</v>
       </c>
     </row>
-    <row r="395" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A395" s="7">
-        <f t="shared" si="6"/>
+    <row r="396" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A396" s="6">
+        <f t="shared" ref="A396:A454" si="6">SUM(A395+1)</f>
         <v>394</v>
       </c>
     </row>
-    <row r="396" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A396" s="7">
+    <row r="397" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A397" s="6">
         <f t="shared" si="6"/>
         <v>395</v>
       </c>
     </row>
-    <row r="397" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A397" s="7">
+    <row r="398" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A398" s="6">
         <f t="shared" si="6"/>
         <v>396</v>
       </c>
     </row>
-    <row r="398" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A398" s="7">
+    <row r="399" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A399" s="6">
         <f t="shared" si="6"/>
         <v>397</v>
       </c>
     </row>
-    <row r="399" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A399" s="7">
+    <row r="400" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A400" s="6">
         <f t="shared" si="6"/>
         <v>398</v>
       </c>
     </row>
-    <row r="400" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A400" s="7">
+    <row r="401" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A401" s="6">
         <f t="shared" si="6"/>
         <v>399</v>
       </c>
     </row>
-    <row r="401" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A401" s="7">
+    <row r="402" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A402" s="6">
         <f t="shared" si="6"/>
         <v>400</v>
       </c>
     </row>
-    <row r="402" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A402" s="7">
+    <row r="403" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A403" s="6">
         <f t="shared" si="6"/>
         <v>401</v>
       </c>
     </row>
-    <row r="403" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A403" s="7">
+    <row r="404" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A404" s="6">
         <f t="shared" si="6"/>
         <v>402</v>
       </c>
     </row>
-    <row r="404" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A404" s="7">
+    <row r="405" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A405" s="6">
         <f t="shared" si="6"/>
         <v>403</v>
       </c>
     </row>
-    <row r="405" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A405" s="7">
+    <row r="406" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A406" s="6">
         <f t="shared" si="6"/>
         <v>404</v>
       </c>
     </row>
-    <row r="406" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A406" s="7">
+    <row r="407" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A407" s="6">
         <f t="shared" si="6"/>
         <v>405</v>
       </c>
     </row>
-    <row r="407" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A407" s="7">
+    <row r="408" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A408" s="6">
         <f t="shared" si="6"/>
         <v>406</v>
       </c>
     </row>
-    <row r="408" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A408" s="7">
+    <row r="409" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A409" s="6">
         <f t="shared" si="6"/>
         <v>407</v>
       </c>
     </row>
-    <row r="409" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A409" s="7">
+    <row r="410" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A410" s="6">
         <f t="shared" si="6"/>
         <v>408</v>
       </c>
     </row>
-    <row r="410" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A410" s="7">
+    <row r="411" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A411" s="6">
         <f t="shared" si="6"/>
         <v>409</v>
       </c>
     </row>
-    <row r="411" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A411" s="7">
+    <row r="412" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A412" s="6">
         <f t="shared" si="6"/>
         <v>410</v>
       </c>
     </row>
-    <row r="412" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A412" s="7">
+    <row r="413" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A413" s="6">
         <f t="shared" si="6"/>
         <v>411</v>
       </c>
     </row>
-    <row r="413" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A413" s="7">
+    <row r="414" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A414" s="6">
         <f t="shared" si="6"/>
         <v>412</v>
       </c>
     </row>
-    <row r="414" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A414" s="7">
+    <row r="415" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A415" s="6">
         <f t="shared" si="6"/>
         <v>413</v>
       </c>
     </row>
-    <row r="415" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A415" s="7">
+    <row r="416" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A416" s="6">
         <f t="shared" si="6"/>
         <v>414</v>
       </c>
     </row>
-    <row r="416" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A416" s="7">
+    <row r="417" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A417" s="6">
         <f t="shared" si="6"/>
         <v>415</v>
       </c>
     </row>
-    <row r="417" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A417" s="7">
+    <row r="418" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A418" s="6">
         <f t="shared" si="6"/>
         <v>416</v>
       </c>
     </row>
-    <row r="418" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A418" s="7">
+    <row r="419" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A419" s="6">
         <f t="shared" si="6"/>
         <v>417</v>
       </c>
     </row>
-    <row r="419" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A419" s="7">
+    <row r="420" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A420" s="6">
         <f t="shared" si="6"/>
         <v>418</v>
       </c>
     </row>
-    <row r="420" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A420" s="7">
+    <row r="421" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A421" s="6">
         <f t="shared" si="6"/>
         <v>419</v>
       </c>
     </row>
-    <row r="421" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A421" s="7">
+    <row r="422" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A422" s="6">
         <f t="shared" si="6"/>
         <v>420</v>
       </c>
     </row>
-    <row r="422" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A422" s="7">
+    <row r="423" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A423" s="6">
         <f t="shared" si="6"/>
         <v>421</v>
       </c>
     </row>
-    <row r="423" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A423" s="7">
+    <row r="424" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A424" s="6">
         <f t="shared" si="6"/>
         <v>422</v>
       </c>
     </row>
-    <row r="424" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A424" s="7">
+    <row r="425" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A425" s="6">
         <f t="shared" si="6"/>
         <v>423</v>
       </c>
     </row>
-    <row r="425" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A425" s="7">
+    <row r="426" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A426" s="6">
         <f t="shared" si="6"/>
         <v>424</v>
       </c>
     </row>
-    <row r="426" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A426" s="7">
+    <row r="427" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A427" s="6">
         <f t="shared" si="6"/>
         <v>425</v>
       </c>
     </row>
-    <row r="427" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A427" s="7">
+    <row r="428" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A428" s="6">
         <f t="shared" si="6"/>
         <v>426</v>
       </c>
     </row>
-    <row r="428" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A428" s="7">
+    <row r="429" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A429" s="6">
         <f t="shared" si="6"/>
         <v>427</v>
       </c>
     </row>
-    <row r="429" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A429" s="7">
+    <row r="430" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A430" s="6">
         <f t="shared" si="6"/>
         <v>428</v>
       </c>
     </row>
-    <row r="430" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A430" s="7">
+    <row r="431" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A431" s="6">
         <f t="shared" si="6"/>
         <v>429</v>
       </c>
     </row>
-    <row r="431" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A431" s="7">
+    <row r="432" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A432" s="6">
         <f t="shared" si="6"/>
         <v>430</v>
       </c>
     </row>
-    <row r="432" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A432" s="7">
+    <row r="433" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A433" s="6">
         <f t="shared" si="6"/>
         <v>431</v>
       </c>
     </row>
-    <row r="433" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A433" s="7">
+    <row r="434" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A434" s="6">
         <f t="shared" si="6"/>
         <v>432</v>
       </c>
     </row>
-    <row r="434" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A434" s="7">
+    <row r="435" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A435" s="6">
         <f t="shared" si="6"/>
         <v>433</v>
       </c>
     </row>
-    <row r="435" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A435" s="7">
+    <row r="436" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A436" s="6">
         <f t="shared" si="6"/>
         <v>434</v>
       </c>
     </row>
-    <row r="436" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A436" s="7">
+    <row r="437" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A437" s="6">
         <f t="shared" si="6"/>
         <v>435</v>
       </c>
     </row>
-    <row r="437" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A437" s="7">
+    <row r="438" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A438" s="6">
         <f t="shared" si="6"/>
         <v>436</v>
       </c>
     </row>
-    <row r="438" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A438" s="7">
+    <row r="439" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A439" s="6">
         <f t="shared" si="6"/>
         <v>437</v>
       </c>
     </row>
-    <row r="439" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A439" s="7">
+    <row r="440" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A440" s="6">
         <f t="shared" si="6"/>
         <v>438</v>
       </c>
     </row>
-    <row r="440" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A440" s="7">
+    <row r="441" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A441" s="6">
         <f t="shared" si="6"/>
         <v>439</v>
       </c>
     </row>
-    <row r="441" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A441" s="7">
+    <row r="442" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A442" s="6">
         <f t="shared" si="6"/>
         <v>440</v>
       </c>
     </row>
-    <row r="442" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A442" s="7">
+    <row r="443" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A443" s="6">
         <f t="shared" si="6"/>
         <v>441</v>
       </c>
     </row>
-    <row r="443" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A443" s="7">
+    <row r="444" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A444" s="6">
         <f t="shared" si="6"/>
         <v>442</v>
       </c>
     </row>
-    <row r="444" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A444" s="7">
+    <row r="445" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A445" s="6">
         <f t="shared" si="6"/>
         <v>443</v>
       </c>
     </row>
-    <row r="445" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A445" s="7">
+    <row r="446" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A446" s="6">
         <f t="shared" si="6"/>
         <v>444</v>
       </c>
     </row>
-    <row r="446" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A446" s="7">
+    <row r="447" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A447" s="6">
         <f t="shared" si="6"/>
         <v>445</v>
       </c>
     </row>
-    <row r="447" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A447" s="7">
+    <row r="448" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A448" s="6">
         <f t="shared" si="6"/>
         <v>446</v>
       </c>
     </row>
-    <row r="448" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A448" s="7">
+    <row r="449" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A449" s="6">
         <f t="shared" si="6"/>
         <v>447</v>
       </c>
     </row>
-    <row r="449" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A449" s="7">
+    <row r="450" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A450" s="6">
         <f t="shared" si="6"/>
         <v>448</v>
       </c>
     </row>
-    <row r="450" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A450" s="7">
+    <row r="451" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A451" s="6">
         <f t="shared" si="6"/>
         <v>449</v>
       </c>
     </row>
-    <row r="451" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A451" s="7">
+    <row r="452" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A452" s="6">
         <f t="shared" si="6"/>
         <v>450</v>
       </c>
     </row>
-    <row r="452" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A452" s="7">
+    <row r="453" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A453" s="6">
         <f t="shared" si="6"/>
         <v>451</v>
+      </c>
+    </row>
+    <row r="454" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A454" s="6">
+        <f t="shared" si="6"/>
+        <v>452</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added some more tests
</commit_message>
<xml_diff>
--- a/documentation/Tests.xlsx
+++ b/documentation/Tests.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://collyer82-my.sharepoint.com/personal/25cookeg899_collyers_ac_uk/Documents/01 - Computer Science/Python Projects/Theatre-Booking/documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="219" documentId="8_{8A25BE57-B96B-4758-82AD-3B4D19E7B08C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E908D8FB-0E5E-4CB0-A919-19C0E4747D78}"/>
+  <xr:revisionPtr revIDLastSave="291" documentId="8_{8A25BE57-B96B-4758-82AD-3B4D19E7B08C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0B66A111-719D-4041-AD02-3D91CAEBA006}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{0216B08E-6C11-4E2A-9B97-BB4BC5AB6A5B}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="177">
   <si>
     <t>Test No</t>
   </si>
@@ -402,6 +402,174 @@
   </si>
   <si>
     <t>Search in search bar</t>
+  </si>
+  <si>
+    <t>Check my bookings redirect works from user dashbaord</t>
+  </si>
+  <si>
+    <t>User is redirected to my bookings page</t>
+  </si>
+  <si>
+    <t>Click my bookings in nav bar</t>
+  </si>
+  <si>
+    <t>Check logout button works in user dashboard</t>
+  </si>
+  <si>
+    <t>Click user name in top right of nav bar</t>
+  </si>
+  <si>
+    <t>User is redirected to main login page</t>
+  </si>
+  <si>
+    <t>Check clicking on a performance works</t>
+  </si>
+  <si>
+    <t>Click on book tickets for a performance</t>
+  </si>
+  <si>
+    <t>User is redireted to select showing page</t>
+  </si>
+  <si>
+    <t>Check select showing works</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Click on a showing </t>
+  </si>
+  <si>
+    <t>User is redirected to seat selection page</t>
+  </si>
+  <si>
+    <t>Check my bookings works from select showing page</t>
+  </si>
+  <si>
+    <t>Click on my bookings in nave bar from select showing page</t>
+  </si>
+  <si>
+    <t>Click on dashboard in nav bar in select showing</t>
+  </si>
+  <si>
+    <t>User is redirected to dashboard</t>
+  </si>
+  <si>
+    <t>Click on user name in top right nav bar of select showing page</t>
+  </si>
+  <si>
+    <t>User is rediretcted to main login page</t>
+  </si>
+  <si>
+    <t>Check logout works from select showing page</t>
+  </si>
+  <si>
+    <t>Check events works from select showings page</t>
+  </si>
+  <si>
+    <t>Check events works from booking page</t>
+  </si>
+  <si>
+    <t>Redirected to main dashboard</t>
+  </si>
+  <si>
+    <t>Check my bookings works from booking page</t>
+  </si>
+  <si>
+    <t>Click on events in booking page</t>
+  </si>
+  <si>
+    <t>Click on my bookings in nav bar of bookings page</t>
+  </si>
+  <si>
+    <t>User redirected to my bookings page</t>
+  </si>
+  <si>
+    <t>Check logout works from booking page</t>
+  </si>
+  <si>
+    <t>Click on username in top right of nav bar in booking page</t>
+  </si>
+  <si>
+    <t>Check booking works with valid data</t>
+  </si>
+  <si>
+    <t>Select three seats and 1 from each age bracket</t>
+  </si>
+  <si>
+    <t>DB is updated and user is redirected to thank you page</t>
+  </si>
+  <si>
+    <t>Check booking works with too few seats</t>
+  </si>
+  <si>
+    <t>Select three seats from and 1 from two of the age brackets</t>
+  </si>
+  <si>
+    <t>Flash message appears and progress stopped</t>
+  </si>
+  <si>
+    <t>Select 2 seats and 1 from eahc age bracket</t>
+  </si>
+  <si>
+    <t>Check events works from thank you page</t>
+  </si>
+  <si>
+    <t>Click events in nav bar of thank you page</t>
+  </si>
+  <si>
+    <t>User si redirected to visitor dashboard</t>
+  </si>
+  <si>
+    <t>Check my bookings works from thank you page</t>
+  </si>
+  <si>
+    <t>Click my bookings in nave bar of thank you page</t>
+  </si>
+  <si>
+    <t>Check log out works from thank you page</t>
+  </si>
+  <si>
+    <t>Click on user name in top right of thank you page</t>
+  </si>
+  <si>
+    <t>Check print tickets works from thank you page</t>
+  </si>
+  <si>
+    <t>Click on print ticket in thank you page</t>
+  </si>
+  <si>
+    <t>PDF ticket with correct data is created and downloaded</t>
+  </si>
+  <si>
+    <t>Check events works from my bookings page</t>
+  </si>
+  <si>
+    <t>Click on events in my bookings page</t>
+  </si>
+  <si>
+    <t>Redirect to user dashboard</t>
+  </si>
+  <si>
+    <t>Check log out works from my bookings page</t>
+  </si>
+  <si>
+    <t>Click on user name in my bookings page</t>
+  </si>
+  <si>
+    <t>Check more details works from thank you page</t>
+  </si>
+  <si>
+    <t>Click on more details for a booking</t>
+  </si>
+  <si>
+    <t>User is redirected to relevent booking thank you page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check book seats works as a special guest </t>
+  </si>
+  <si>
+    <t>Book seast as a special account</t>
+  </si>
+  <si>
+    <t>Price is £0.00</t>
   </si>
 </sst>
 </file>
@@ -459,7 +627,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -482,7 +650,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1341,7 +1508,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="33" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A33" s="6">
         <f t="shared" si="0"/>
         <v>32</v>
@@ -1356,7 +1523,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="34" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A34" s="6">
         <f t="shared" si="0"/>
         <v>33</v>
@@ -1371,7 +1538,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="35" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A35" s="6">
         <f t="shared" si="0"/>
         <v>34</v>
@@ -1386,7 +1553,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="36" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A36" s="6">
         <f t="shared" si="0"/>
         <v>35</v>
@@ -1401,7 +1568,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="37" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A37" s="6">
         <f t="shared" si="0"/>
         <v>36</v>
@@ -1416,7 +1583,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="38" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A38" s="6">
         <f t="shared" si="0"/>
         <v>37</v>
@@ -1431,7 +1598,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="39" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A39" s="6">
         <f t="shared" si="0"/>
         <v>38</v>
@@ -1446,7 +1613,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="40" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A40" s="6">
         <f t="shared" si="0"/>
         <v>39</v>
@@ -1461,7 +1628,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="41" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A41" s="6">
         <f t="shared" si="0"/>
         <v>40</v>
@@ -1476,7 +1643,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="42" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A42" s="6">
         <v>40</v>
       </c>
@@ -1490,7 +1657,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="43" spans="1:6" s="8" customFormat="1" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:4" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="6">
         <v>41</v>
       </c>
@@ -1503,9 +1670,8 @@
       <c r="D43" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="F43" s="5"/>
-    </row>
-    <row r="44" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="44" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A44" s="6">
         <f>SUM(A43+1)</f>
         <v>42</v>
@@ -1520,7 +1686,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="45" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A45" s="6">
         <f t="shared" si="0"/>
         <v>43</v>
@@ -1535,7 +1701,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="46" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A46" s="6">
         <f t="shared" si="0"/>
         <v>44</v>
@@ -1550,7 +1716,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="47" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A47" s="6">
         <f t="shared" si="0"/>
         <v>45</v>
@@ -1565,199 +1731,388 @@
         <v>118</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A48" s="6">
         <f t="shared" si="0"/>
         <v>46</v>
       </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B48" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A49" s="6">
         <f t="shared" si="0"/>
         <v>47</v>
       </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B49" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="D49" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A50" s="6">
         <f t="shared" si="0"/>
         <v>48</v>
       </c>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B50" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A51" s="6">
         <f t="shared" si="0"/>
         <v>49</v>
       </c>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B51" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="D51" s="1" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A52" s="6">
         <f t="shared" si="0"/>
         <v>50</v>
       </c>
-    </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B52" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A53" s="6">
         <f t="shared" si="0"/>
         <v>51</v>
       </c>
-    </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B53" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="D53" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A54" s="6">
         <f t="shared" si="0"/>
         <v>52</v>
       </c>
-    </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B54" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A55" s="6">
         <f t="shared" si="0"/>
         <v>53</v>
       </c>
-    </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B55" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A56" s="6">
         <f t="shared" si="0"/>
         <v>54</v>
       </c>
-    </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B56" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D56" s="1" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A57" s="6">
         <f t="shared" si="0"/>
         <v>55</v>
       </c>
-    </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B57" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="D57" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A58" s="6">
         <f t="shared" si="0"/>
         <v>56</v>
       </c>
-    </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B58" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="D58" s="1" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A59" s="6">
         <f t="shared" si="0"/>
         <v>57</v>
       </c>
-    </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B59" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="D59" s="1" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A60" s="6">
         <f t="shared" si="0"/>
         <v>58</v>
       </c>
-    </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B60" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="D60" s="1" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A61" s="6">
         <f t="shared" si="0"/>
         <v>59</v>
       </c>
-    </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B61" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D61" s="1" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A62" s="6">
         <f t="shared" si="0"/>
         <v>60</v>
       </c>
-    </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B62" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="D62" s="1" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A63" s="6">
         <f t="shared" si="0"/>
         <v>61</v>
       </c>
-    </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B63" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="D63" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A64" s="6">
         <f t="shared" si="0"/>
         <v>62</v>
       </c>
-    </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B64" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="D64" s="1" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A65" s="6">
         <f t="shared" si="0"/>
         <v>63</v>
       </c>
-    </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B65" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="D65" s="1" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A66" s="6">
         <f t="shared" si="0"/>
         <v>64</v>
       </c>
-    </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B66" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="D66" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A67" s="6">
         <f t="shared" si="0"/>
         <v>65</v>
       </c>
-    </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B67" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="D67" s="1" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A68" s="6">
         <f t="shared" si="0"/>
         <v>66</v>
       </c>
-    </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B68" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="C68" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="D68" s="1" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A69" s="6">
         <f t="shared" si="0"/>
         <v>67</v>
       </c>
     </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A70" s="6">
         <f t="shared" si="0"/>
         <v>68</v>
       </c>
     </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A71" s="6">
         <f t="shared" si="0"/>
         <v>69</v>
       </c>
     </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A72" s="6">
         <f t="shared" si="0"/>
         <v>70</v>
       </c>
     </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A73" s="6">
         <f t="shared" si="0"/>
         <v>71</v>
       </c>
     </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A74" s="6">
         <f t="shared" si="0"/>
         <v>72</v>
       </c>
     </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A75" s="6">
         <f t="shared" si="0"/>
         <v>73</v>
       </c>
     </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A76" s="6">
         <f t="shared" ref="A76:A139" si="1">SUM(A75+1)</f>
         <v>74</v>
       </c>
     </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A77" s="6">
         <f t="shared" si="1"/>
         <v>75</v>
       </c>
     </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A78" s="6">
         <f t="shared" si="1"/>
         <v>76</v>
       </c>
     </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A79" s="6">
         <f t="shared" si="1"/>
         <v>77</v>
       </c>
     </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A80" s="6">
         <f t="shared" si="1"/>
         <v>78</v>

</xml_diff>